<commit_message>
Checklist: event-name title row; columns 번호/물품/확인1/확인2/비고 (O/X)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GKZaWMuKZZscZ9zMq94jVY
</commit_message>
<xml_diff>
--- a/체크리스트.xlsx
+++ b/체크리스트.xlsx
@@ -10,7 +10,7 @@
     <sheet name="체크리스트" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'체크리스트'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'체크리스트'!$1:$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,13 +19,17 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="18"/>
     </font>
     <font>
       <b val="1"/>
@@ -46,13 +50,18 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="004472C4"/>
+      </bottom>
     </border>
     <border>
       <left style="thin">
@@ -72,16 +81,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -472,495 +484,505 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
+    <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>행사명</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>번호</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>물품</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>확인1</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>확인2</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>확인3</t>
+          <t>비고</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="3" t="n">
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="2" t="n"/>
-      <c r="B3" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="B3" s="4" t="n"/>
       <c r="C3" s="3" t="n"/>
       <c r="D3" s="3" t="n"/>
       <c r="E3" s="3" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="A4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="n"/>
       <c r="C4" s="3" t="n"/>
       <c r="D4" s="3" t="n"/>
       <c r="E4" s="3" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="2" t="n"/>
-      <c r="B5" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4" t="n"/>
       <c r="C5" s="3" t="n"/>
       <c r="D5" s="3" t="n"/>
       <c r="E5" s="3" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="A6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4" t="n"/>
       <c r="C6" s="3" t="n"/>
       <c r="D6" s="3" t="n"/>
       <c r="E6" s="3" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="3" t="n">
-        <v>6</v>
-      </c>
+      <c r="A7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="4" t="n"/>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="3" t="n"/>
       <c r="E7" s="3" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="3" t="n">
-        <v>7</v>
-      </c>
+      <c r="A8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="4" t="n"/>
       <c r="C8" s="3" t="n"/>
       <c r="D8" s="3" t="n"/>
       <c r="E8" s="3" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="2" t="n"/>
-      <c r="B9" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="A9" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="4" t="n"/>
       <c r="C9" s="3" t="n"/>
       <c r="D9" s="3" t="n"/>
       <c r="E9" s="3" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="2" t="n"/>
-      <c r="B10" s="3" t="n">
-        <v>9</v>
-      </c>
+      <c r="A10" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="4" t="n"/>
       <c r="C10" s="3" t="n"/>
       <c r="D10" s="3" t="n"/>
       <c r="E10" s="3" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="2" t="n"/>
-      <c r="B11" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="A11" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="4" t="n"/>
       <c r="C11" s="3" t="n"/>
       <c r="D11" s="3" t="n"/>
       <c r="E11" s="3" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="3" t="n">
-        <v>11</v>
-      </c>
+      <c r="A12" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="4" t="n"/>
       <c r="C12" s="3" t="n"/>
       <c r="D12" s="3" t="n"/>
       <c r="E12" s="3" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="2" t="n"/>
-      <c r="B13" s="3" t="n">
-        <v>12</v>
-      </c>
+      <c r="A13" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="4" t="n"/>
       <c r="C13" s="3" t="n"/>
       <c r="D13" s="3" t="n"/>
       <c r="E13" s="3" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="2" t="n"/>
-      <c r="B14" s="3" t="n">
-        <v>13</v>
-      </c>
+      <c r="A14" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="4" t="n"/>
       <c r="C14" s="3" t="n"/>
       <c r="D14" s="3" t="n"/>
       <c r="E14" s="3" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="2" t="n"/>
-      <c r="B15" s="3" t="n">
-        <v>14</v>
-      </c>
+      <c r="A15" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="4" t="n"/>
       <c r="C15" s="3" t="n"/>
       <c r="D15" s="3" t="n"/>
       <c r="E15" s="3" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="3" t="n">
-        <v>15</v>
-      </c>
+      <c r="A16" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="4" t="n"/>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="3" t="n"/>
       <c r="E16" s="3" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="2" t="n"/>
-      <c r="B17" s="3" t="n">
-        <v>16</v>
-      </c>
+      <c r="A17" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="4" t="n"/>
       <c r="C17" s="3" t="n"/>
       <c r="D17" s="3" t="n"/>
       <c r="E17" s="3" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="2" t="n"/>
-      <c r="B18" s="3" t="n">
-        <v>17</v>
-      </c>
+      <c r="A18" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="4" t="n"/>
       <c r="C18" s="3" t="n"/>
       <c r="D18" s="3" t="n"/>
       <c r="E18" s="3" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="3" t="n">
-        <v>18</v>
-      </c>
+      <c r="A19" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="4" t="n"/>
       <c r="C19" s="3" t="n"/>
       <c r="D19" s="3" t="n"/>
       <c r="E19" s="3" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="2" t="n"/>
-      <c r="B20" s="3" t="n">
-        <v>19</v>
-      </c>
+      <c r="A20" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="4" t="n"/>
       <c r="C20" s="3" t="n"/>
       <c r="D20" s="3" t="n"/>
       <c r="E20" s="3" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="2" t="n"/>
-      <c r="B21" s="3" t="n">
-        <v>20</v>
-      </c>
+      <c r="A21" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="4" t="n"/>
       <c r="C21" s="3" t="n"/>
       <c r="D21" s="3" t="n"/>
       <c r="E21" s="3" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="2" t="n"/>
-      <c r="B22" s="3" t="n">
-        <v>21</v>
-      </c>
+      <c r="A22" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="4" t="n"/>
       <c r="C22" s="3" t="n"/>
       <c r="D22" s="3" t="n"/>
       <c r="E22" s="3" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="2" t="n"/>
-      <c r="B23" s="3" t="n">
-        <v>22</v>
-      </c>
+      <c r="A23" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="4" t="n"/>
       <c r="C23" s="3" t="n"/>
       <c r="D23" s="3" t="n"/>
       <c r="E23" s="3" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="3" t="n">
-        <v>23</v>
-      </c>
+      <c r="A24" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="4" t="n"/>
       <c r="C24" s="3" t="n"/>
       <c r="D24" s="3" t="n"/>
       <c r="E24" s="3" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="3" t="n">
-        <v>24</v>
-      </c>
+      <c r="A25" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="4" t="n"/>
       <c r="C25" s="3" t="n"/>
       <c r="D25" s="3" t="n"/>
       <c r="E25" s="3" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="3" t="n">
-        <v>25</v>
-      </c>
+      <c r="A26" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="4" t="n"/>
       <c r="C26" s="3" t="n"/>
       <c r="D26" s="3" t="n"/>
       <c r="E26" s="3" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="2" t="n"/>
-      <c r="B27" s="3" t="n">
-        <v>26</v>
-      </c>
+      <c r="A27" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="4" t="n"/>
       <c r="C27" s="3" t="n"/>
       <c r="D27" s="3" t="n"/>
       <c r="E27" s="3" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="2" t="n"/>
-      <c r="B28" s="3" t="n">
-        <v>27</v>
-      </c>
+      <c r="A28" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" s="4" t="n"/>
       <c r="C28" s="3" t="n"/>
       <c r="D28" s="3" t="n"/>
       <c r="E28" s="3" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="2" t="n"/>
-      <c r="B29" s="3" t="n">
-        <v>28</v>
-      </c>
+      <c r="A29" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="4" t="n"/>
       <c r="C29" s="3" t="n"/>
       <c r="D29" s="3" t="n"/>
       <c r="E29" s="3" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="2" t="n"/>
-      <c r="B30" s="3" t="n">
-        <v>29</v>
-      </c>
+      <c r="A30" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="4" t="n"/>
       <c r="C30" s="3" t="n"/>
       <c r="D30" s="3" t="n"/>
       <c r="E30" s="3" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="2" t="n"/>
-      <c r="B31" s="3" t="n">
-        <v>30</v>
-      </c>
+      <c r="A31" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" s="4" t="n"/>
       <c r="C31" s="3" t="n"/>
       <c r="D31" s="3" t="n"/>
       <c r="E31" s="3" t="n"/>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="2" t="n"/>
-      <c r="B32" s="3" t="n">
-        <v>31</v>
-      </c>
+      <c r="A32" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" s="4" t="n"/>
       <c r="C32" s="3" t="n"/>
       <c r="D32" s="3" t="n"/>
       <c r="E32" s="3" t="n"/>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="2" t="n"/>
-      <c r="B33" s="3" t="n">
-        <v>32</v>
-      </c>
+      <c r="A33" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" s="4" t="n"/>
       <c r="C33" s="3" t="n"/>
       <c r="D33" s="3" t="n"/>
       <c r="E33" s="3" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="2" t="n"/>
-      <c r="B34" s="3" t="n">
-        <v>33</v>
-      </c>
+      <c r="A34" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" s="4" t="n"/>
       <c r="C34" s="3" t="n"/>
       <c r="D34" s="3" t="n"/>
       <c r="E34" s="3" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="2" t="n"/>
-      <c r="B35" s="3" t="n">
-        <v>34</v>
-      </c>
+      <c r="A35" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" s="4" t="n"/>
       <c r="C35" s="3" t="n"/>
       <c r="D35" s="3" t="n"/>
       <c r="E35" s="3" t="n"/>
     </row>
     <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="2" t="n"/>
-      <c r="B36" s="3" t="n">
-        <v>35</v>
-      </c>
+      <c r="A36" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" s="4" t="n"/>
       <c r="C36" s="3" t="n"/>
       <c r="D36" s="3" t="n"/>
       <c r="E36" s="3" t="n"/>
     </row>
     <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="2" t="n"/>
-      <c r="B37" s="3" t="n">
-        <v>36</v>
-      </c>
+      <c r="A37" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" s="4" t="n"/>
       <c r="C37" s="3" t="n"/>
       <c r="D37" s="3" t="n"/>
       <c r="E37" s="3" t="n"/>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="2" t="n"/>
-      <c r="B38" s="3" t="n">
-        <v>37</v>
-      </c>
+      <c r="A38" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" s="4" t="n"/>
       <c r="C38" s="3" t="n"/>
       <c r="D38" s="3" t="n"/>
       <c r="E38" s="3" t="n"/>
     </row>
     <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="2" t="n"/>
-      <c r="B39" s="3" t="n">
-        <v>38</v>
-      </c>
+      <c r="A39" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" s="4" t="n"/>
       <c r="C39" s="3" t="n"/>
       <c r="D39" s="3" t="n"/>
       <c r="E39" s="3" t="n"/>
     </row>
     <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="2" t="n"/>
-      <c r="B40" s="3" t="n">
-        <v>39</v>
-      </c>
+      <c r="A40" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" s="4" t="n"/>
       <c r="C40" s="3" t="n"/>
       <c r="D40" s="3" t="n"/>
       <c r="E40" s="3" t="n"/>
     </row>
     <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="2" t="n"/>
-      <c r="B41" s="3" t="n">
-        <v>40</v>
-      </c>
+      <c r="A41" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" s="4" t="n"/>
       <c r="C41" s="3" t="n"/>
       <c r="D41" s="3" t="n"/>
       <c r="E41" s="3" t="n"/>
     </row>
     <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="2" t="n"/>
-      <c r="B42" s="3" t="n">
-        <v>41</v>
-      </c>
+      <c r="A42" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" s="4" t="n"/>
       <c r="C42" s="3" t="n"/>
       <c r="D42" s="3" t="n"/>
       <c r="E42" s="3" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="2" t="n"/>
-      <c r="B43" s="3" t="n">
-        <v>42</v>
-      </c>
+      <c r="A43" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" s="4" t="n"/>
       <c r="C43" s="3" t="n"/>
       <c r="D43" s="3" t="n"/>
       <c r="E43" s="3" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="2" t="n"/>
-      <c r="B44" s="3" t="n">
-        <v>43</v>
-      </c>
+      <c r="A44" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" s="4" t="n"/>
       <c r="C44" s="3" t="n"/>
       <c r="D44" s="3" t="n"/>
       <c r="E44" s="3" t="n"/>
     </row>
     <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="2" t="n"/>
-      <c r="B45" s="3" t="n">
-        <v>44</v>
-      </c>
+      <c r="A45" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" s="4" t="n"/>
       <c r="C45" s="3" t="n"/>
       <c r="D45" s="3" t="n"/>
       <c r="E45" s="3" t="n"/>
     </row>
     <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="2" t="n"/>
-      <c r="B46" s="3" t="n">
-        <v>45</v>
-      </c>
+      <c r="A46" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" s="4" t="n"/>
       <c r="C46" s="3" t="n"/>
       <c r="D46" s="3" t="n"/>
       <c r="E46" s="3" t="n"/>
     </row>
     <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="2" t="n"/>
-      <c r="B47" s="3" t="n">
-        <v>46</v>
-      </c>
+      <c r="A47" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" s="4" t="n"/>
       <c r="C47" s="3" t="n"/>
       <c r="D47" s="3" t="n"/>
       <c r="E47" s="3" t="n"/>
     </row>
     <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="2" t="n"/>
-      <c r="B48" s="3" t="n">
-        <v>47</v>
-      </c>
+      <c r="A48" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" s="4" t="n"/>
       <c r="C48" s="3" t="n"/>
       <c r="D48" s="3" t="n"/>
       <c r="E48" s="3" t="n"/>
     </row>
     <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="2" t="n"/>
-      <c r="B49" s="3" t="n">
-        <v>48</v>
-      </c>
+      <c r="A49" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" s="4" t="n"/>
       <c r="C49" s="3" t="n"/>
       <c r="D49" s="3" t="n"/>
       <c r="E49" s="3" t="n"/>
     </row>
     <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="2" t="n"/>
-      <c r="B50" s="3" t="n">
-        <v>49</v>
-      </c>
+      <c r="A50" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" s="4" t="n"/>
       <c r="C50" s="3" t="n"/>
       <c r="D50" s="3" t="n"/>
       <c r="E50" s="3" t="n"/>
     </row>
     <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="2" t="n"/>
-      <c r="B51" s="3" t="n">
-        <v>50</v>
-      </c>
+      <c r="A51" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" s="4" t="n"/>
       <c r="C51" s="3" t="n"/>
       <c r="D51" s="3" t="n"/>
       <c r="E51" s="3" t="n"/>
     </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" s="4" t="n"/>
+      <c r="C52" s="3" t="n"/>
+      <c r="D52" s="3" t="n"/>
+      <c r="E52" s="3" t="n"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C2:E51">
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C3:E52">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"O"</formula>
     </cfRule>
@@ -969,7 +991,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="C2:E51" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="입력 오류" error="O 또는 X만 입력하세요." type="list">
+    <dataValidation sqref="C3:E52" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="입력 오류" error="O 또는 X만 입력하세요." type="list">
       <formula1>"O,X"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>